<commit_message>
fix/feat: correct hyperlink target for Beispiel warranty link in all templates and regenerate supplier files
</commit_message>
<xml_diff>
--- a/Meilenstein 1/Lieferantenabfrage/Supplier_Warranty_Inquiry_Template_DE.xlsx
+++ b/Meilenstein 1/Lieferantenabfrage/Supplier_Warranty_Inquiry_Template_DE.xlsx
@@ -1,136 +1,57 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\thomas.winkler\Desktop\Projekte\Google Antigravity\ELEKTROPEPI\GEWAEHRLEISTUNG_GARANTIELABEL\Meilenstein 1\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{81EBD72D-324C-45F5-B67F-62BCC659C31A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Beispiel" sheetId="1" r:id="rId1"/>
-    <sheet name="Garantiedaten_Erfassung" sheetId="2" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Beispiel" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Garantiedaten_Erfassung" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <definedNames/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="23">
-  <si>
-    <t>Feld-Attribut / Spalte</t>
-  </si>
-  <si>
-    <t>Ausfüllbeispiel für einen Musterartikel</t>
-  </si>
-  <si>
-    <t>Begründung / Gesetzliche Grundlage (Warum wird das benötigt?)</t>
-  </si>
-  <si>
-    <t>EAN / GTIN (Barcode)</t>
-  </si>
-  <si>
-    <t>4895251607063</t>
-  </si>
-  <si>
-    <t>Dient der eindeutigen und automatisierten Produktzuordnung in der SBS-Datenbank. Ohne EAN ist kein automatischer Import möglich.</t>
-  </si>
-  <si>
-    <t>Lieferanten-Artikelnummer (Herstellernummer)</t>
-  </si>
-  <si>
-    <t>EF BD-5.1-S1</t>
-  </si>
-  <si>
-    <t>Dient als Ersatzschlüssel zur Zuordnung und erleichtert die eindeutige Identifikation bei Rückfragen oder Datenfehlern.</t>
-  </si>
-  <si>
-    <t>Marke / Brand</t>
-  </si>
-  <si>
-    <t>EcoFlow</t>
-  </si>
-  <si>
-    <t>Gesetzliches Pflichtfeld („Brand/Trademark“) laut Durchführungsverordnung (EU) 2025/1960. Wird direkt auf dem Garantielabel abgedruckt.</t>
-  </si>
-  <si>
-    <t>Modellkennung / Model identifier</t>
-  </si>
-  <si>
-    <t>PowerOcean LFP Batterie (5 kWh)</t>
-  </si>
-  <si>
-    <t>Gesetzliches Pflichtfeld („Model identifier“) laut Durchführungsverordnung (EU) 2025/1960. Muss exakt mit den Angaben auf dem Produkt übereinstimmen.</t>
-  </si>
-  <si>
-    <t>Garantiedauer in Jahren (XX)</t>
-  </si>
-  <si>
-    <t>Gesetzliches Pflichtfeld laut Durchführungsverordnung (EU) 2025/1960. Bestimmt den aufgedruckten Garantiewert (Jahre &gt; 2) auf dem EU-Label.</t>
-  </si>
-  <si>
-    <t>Link zu den Garantiebedingungen</t>
-  </si>
-  <si>
-    <t>https://enterprise-service-eu-cdn.ecoflow.com/enterprise/documentation/1719480779438/20240627EcoFlow%20Warranty%20Policy%20for%20Home%20Solar%20Battery%20Solutions%20in%20Europe%20B%20V1.3-EN.pdf</t>
-  </si>
-  <si>
-    <t>Gesetzlich zwingend nach § 9a Abs 3 KSchG. Die Garantieerklärung muss dem Verbraucher auf einem dauerhaften Datenträger (z. B. per PDF-Link) bereitgestellt werden.</t>
-  </si>
-  <si>
-    <t>Bestätigung 'Kostenlose Vollgarantie' (Ja/Nein)</t>
-  </si>
-  <si>
-    <t>Ja</t>
-  </si>
-  <si>
-    <t>Rechtliche Absicherung für SBS. Das grüne EU-Garantielabel darf ausschließlich für kostenlose Vollgarantien genutzt werden (Vermeidung von Abmahnungen).</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
+  <fonts count="5">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="FFFFFFFF"/>
       <sz val="12"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Calibri"/>
     </font>
     <font>
-      <b/>
+      <name val="Calibri"/>
+      <b val="1"/>
       <sz val="11"/>
-      <name val="Calibri"/>
     </font>
     <font>
+      <name val="Calibri"/>
       <sz val="11"/>
-      <name val="Calibri"/>
     </font>
     <font>
-      <u/>
-      <sz val="11"/>
-      <color theme="10"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <color theme="10"/>
+      <sz val="11"/>
+      <u val="single"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="4">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -207,58 +128,117 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="9">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
+    <cellStyle name="Standard" xfId="0" builtinId="0"/>
     <cellStyle name="Link" xfId="1" builtinId="8"/>
-    <cellStyle name="Standard" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Tabelle1" displayName="Tabelle1" ref="A1:G2" totalsRowShown="0">
-  <autoFilter ref="A1:G2" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Tabelle1" displayName="Tabelle1" ref="A1:G2" headerRowCount="1" totalsRowShown="0">
+  <autoFilter ref="A1:G2"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="EAN / GTIN (Barcode)"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Lieferanten-Artikelnummer (Herstellernummer)"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Marke / Brand"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Modellkennung / Model identifier"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Garantiedauer in Jahren (XX)"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="Link zu den Garantiebedingungen"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="Bestätigung 'Kostenlose Vollgarantie' (Ja/Nein)"/>
+    <tableColumn id="1" name="EAN / GTIN (Barcode)"/>
+    <tableColumn id="2" name="Lieferanten-Artikelnummer (Herstellernummer)"/>
+    <tableColumn id="3" name="Marke / Brand"/>
+    <tableColumn id="4" name="Modellkennung / Model identifier"/>
+    <tableColumn id="5" name="Garantiedauer in Jahren (XX)"/>
+    <tableColumn id="6" name="Link zu den Garantiebedingungen"/>
+    <tableColumn id="7" name="Bestätigung 'Kostenlose Vollgarantie' (Ja/Nein)"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -548,163 +528,231 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C9"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C8"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="45" customWidth="1"/>
-    <col min="2" max="2" width="65" customWidth="1"/>
-    <col min="3" max="3" width="77.5703125" customWidth="1"/>
+    <col width="45" customWidth="1" min="1" max="1"/>
+    <col width="65" customWidth="1" min="2" max="2"/>
+    <col width="77.5703125" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="7" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="B2" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="C2" s="8" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="B3" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="C3" s="8" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="C4" s="8" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="B5" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="C5" s="8" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="4" t="s">
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Feld-Attribut / Spalte</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Ausfüllbeispiel für einen Musterartikel</t>
+        </is>
+      </c>
+      <c r="C1" s="7" t="inlineStr">
+        <is>
+          <t>Begründung / Gesetzliche Grundlage (Warum wird das benötigt?)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="39.95" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>EAN / GTIN (Barcode)</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>4895251607063</t>
+        </is>
+      </c>
+      <c r="C2" s="8" t="inlineStr">
+        <is>
+          <t>Dient der eindeutigen und automatisierten Produktzuordnung in der SBS-Datenbank. Ohne EAN ist kein automatischer Import möglich.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="39.95" customHeight="1">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Lieferanten-Artikelnummer (Herstellernummer)</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>EF BD-5.1-S1</t>
+        </is>
+      </c>
+      <c r="C3" s="8" t="inlineStr">
+        <is>
+          <t>Dient als Ersatzschlüssel zur Zuordnung und erleichtert die eindeutige Identifikation bei Rückfragen oder Datenfehlern.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="39.95" customHeight="1">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Marke / Brand</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>EcoFlow</t>
+        </is>
+      </c>
+      <c r="C4" s="8" t="inlineStr">
+        <is>
+          <t>Gesetzliches Pflichtfeld („Brand/Trademark“) laut Durchführungsverordnung (EU) 2025/1960. Wird direkt auf dem Garantielabel abgedruckt.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="39.95" customHeight="1">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Modellkennung / Model identifier</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>PowerOcean LFP Batterie (5 kWh)</t>
+        </is>
+      </c>
+      <c r="C5" s="8" t="inlineStr">
+        <is>
+          <t>Gesetzliches Pflichtfeld („Model identifier“) laut Durchführungsverordnung (EU) 2025/1960. Muss exakt mit den Angaben auf dem Produkt übereinstimmen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="39.95" customHeight="1">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Garantiedauer in Jahren (XX)</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
         <v>15</v>
       </c>
-      <c r="B6" s="5">
-        <v>15</v>
-      </c>
-      <c r="C6" s="8" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" ht="69.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="B7" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="C7" s="8" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="B8" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="C8" s="8" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25"/>
+      <c r="C6" s="8" t="inlineStr">
+        <is>
+          <t>Gesetzliches Pflichtfeld laut Durchführungsverordnung (EU) 2025/1960. Bestimmt den aufgedruckten Garantiewert (Jahre &gt; 2) auf dem EU-Label.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="69.75" customHeight="1">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Link zu den Garantiebedingungen</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>https://enterprise-service-eu-cdn.ecoflow.com/enterprise/documentation/1719480779438/20240627EcoFlow%20Warranty%20Policy%20for%20Home%20Solar%20Battery%20Solutions%20in%20Europe%20B%20V1.3-EN.pdf</t>
+        </is>
+      </c>
+      <c r="C7" s="8" t="inlineStr">
+        <is>
+          <t>Gesetzlich zwingend nach § 9a Abs 3 KSchG. Die Garantieerklärung muss dem Verbraucher auf einem dauerhaften Datenträger (z. B. per PDF-Link) bereitgestellt werden.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="39.95" customHeight="1">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>Bestätigung 'Kostenlose Vollgarantie' (Ja/Nein)</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="C8" s="8" t="inlineStr">
+        <is>
+          <t>Rechtliche Absicherung für SBS. Das grüne EU-Garantielabel darf ausschließlich für kostenlose Vollgarantien genutzt werden (Vermeidung von Abmahnungen).</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="21.95" customHeight="1"/>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="B7" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B7" r:id="rId1"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:G1"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="25" customWidth="1"/>
-    <col min="2" max="4" width="30" customWidth="1"/>
-    <col min="5" max="5" width="25" customWidth="1"/>
-    <col min="6" max="6" width="45" customWidth="1"/>
-    <col min="7" max="7" width="35" customWidth="1"/>
-    <col min="8" max="8" width="10" customWidth="1"/>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="4"/>
+    <col width="25" customWidth="1" min="5" max="5"/>
+    <col width="45" customWidth="1" min="6" max="6"/>
+    <col width="35" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B1" t="s">
-        <v>6</v>
-      </c>
-      <c r="C1" t="s">
-        <v>9</v>
-      </c>
-      <c r="D1" t="s">
-        <v>12</v>
-      </c>
-      <c r="E1" t="s">
-        <v>15</v>
-      </c>
-      <c r="F1" t="s">
-        <v>17</v>
-      </c>
-      <c r="G1" t="s">
-        <v>20</v>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>EAN / GTIN (Barcode)</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Lieferanten-Artikelnummer (Herstellernummer)</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Marke / Brand</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Modellkennung / Model identifier</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Garantiedauer in Jahren (XX)</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Link zu den Garantiebedingungen</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Bestätigung 'Kostenlose Vollgarantie' (Ja/Nein)</t>
+        </is>
       </c>
     </row>
   </sheetData>
   <dataValidations count="5">
-    <dataValidation promptTitle="Marke / Brand" prompt="Tragen Sie bitte den kurzen Markennamen ein, der auf dem Label stehen soll (z. B. „Miele“ statt „Miele GmbH“)." sqref="C2:C1000" xr:uid="{00000000-0002-0000-0100-000000000000}"/>
-    <dataValidation promptTitle="Modellbezeichnung" prompt="Tragen Sie bitte die exakte Modellkennung des Herstellers ein (z. B. „WXD160“)." sqref="D2:D1000" xr:uid="{00000000-0002-0000-0100-000001000000}"/>
-    <dataValidation type="whole" operator="greaterThan" errorTitle="Ungültiger Wert" error="Geben Sie bitte eine ganze Zahl größer als 2 ein (z.B. 3, 5, 10)." promptTitle="Herstellergarantie" prompt="Tragen Sie hier bitte ausschließlich die nackte Zahl ein (z. B. 3, 5, 10). Schreiben Sie keine Einheiten wie „Jahre“ oder „J“ dazu." sqref="E2:E1000" xr:uid="{00000000-0002-0000-0100-000002000000}">
+    <dataValidation sqref="C2:C1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" promptTitle="Marke / Brand" prompt="Tragen Sie bitte den kurzen Markennamen ein, der auf dem Label stehen soll (z. B. „Miele“ statt „Miele GmbH“)."/>
+    <dataValidation sqref="D2:D1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" promptTitle="Modellbezeichnung" prompt="Tragen Sie bitte die exakte Modellkennung des Herstellers ein (z. B. „WXD160“)."/>
+    <dataValidation sqref="E2:E1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Ungültiger Wert" error="Geben Sie bitte eine ganze Zahl größer als 2 ein (z.B. 3, 5, 10)." promptTitle="Herstellergarantie" prompt="Tragen Sie hier bitte ausschließlich die nackte Zahl ein (z. B. 3, 5, 10). Schreiben Sie keine Einheiten wie „Jahre“ oder „J“ dazu." type="whole" operator="greaterThan">
       <formula1>2</formula1>
     </dataValidation>
-    <dataValidation promptTitle="Link zu Garantiebedingungen" prompt="Bitte tragen Sie hier den direkten Link (URL) zu den Garantiebedingungen auf Ihrer Website ein (z. B. https://www.hersteller.at/garantie). Schreiben Sie keinen Freitext wie „liegt bei“." sqref="F2:F1000" xr:uid="{00000000-0002-0000-0100-000003000000}"/>
-    <dataValidation type="list" errorTitle="Ungültige Auswahl" error="Ungültige Auswahl. Bitte wählen Sie Ja oder Nein aus dem Dropdown-Menü." promptTitle="Garantie-Bestätigung" prompt="Bitte wählen Sie ausschließlich „Ja“ oder „Nein“ aus dem Dropdown-Menü aus." sqref="G2:G1000" xr:uid="{00000000-0002-0000-0100-000004000000}">
+    <dataValidation sqref="F2:F1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" promptTitle="Link zu Garantiebedingungen" prompt="Bitte tragen Sie hier den direkten Link (URL) zu den Garantiebedingungen auf Ihrer Website ein (z. B. https://www.hersteller.at/garantie). Schreiben Sie keinen Freitext wie „liegt bei“."/>
+    <dataValidation sqref="G2:G1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Ungültige Auswahl" error="Ungültige Auswahl. Bitte wählen Sie Ja oder Nein aus dem Dropdown-Menü." promptTitle="Garantie-Bestätigung" prompt="Bitte wählen Sie ausschließlich „Ja“ oder „Nein“ aus dem Dropdown-Menü aus." type="list">
       <formula1>"Ja,Nein"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
-    <tablePart r:id="rId1"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>